<commit_message>
Actualizacion de datos en Excel
</commit_message>
<xml_diff>
--- a/ventas_ficticias_Q1_2026.xlsx
+++ b/ventas_ficticias_Q1_2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\INFORMATICA\Desktop\prueba\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDC39307-ACE2-4A26-B04E-F9748792EF83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20DCF9D4-12CD-4938-9813-FDD1EE14CA7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="31">
   <si>
     <t>Concepto</t>
   </si>
@@ -2266,12 +2266,12 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7875F631-FE92-4E7E-8946-FDF27C28EBB3}">
-  <dimension ref="A1:D41"/>
+  <dimension ref="A1:D42"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31.5703125" customWidth="1"/>
     <col min="2" max="2" width="22.7109375" style="9" customWidth="1"/>
-    <col min="3" max="3" width="18.28515625" customWidth="1"/>
+    <col min="3" max="3" width="16.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -2848,6 +2848,16 @@
         <v>7</v>
       </c>
     </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B42"/>
+      <c r="C42" s="6">
+        <f>SUM(C2:C41)</f>
+        <v>106240.79999999999</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Ajuste de nombre de columna Monto en dolares
</commit_message>
<xml_diff>
--- a/ventas_ficticias_Q1_2026.xlsx
+++ b/ventas_ficticias_Q1_2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\INFORMATICA\Desktop\prueba\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20DCF9D4-12CD-4938-9813-FDD1EE14CA7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2B6567C-64F7-4F5A-A6C1-9AF274914CB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2271,7 +2271,7 @@
   <cols>
     <col min="1" max="1" width="31.5703125" customWidth="1"/>
     <col min="2" max="2" width="22.7109375" style="9" customWidth="1"/>
-    <col min="3" max="3" width="16.28515625" customWidth="1"/>
+    <col min="3" max="3" width="20.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Lectura de todas las pestañas del Excel y filtro de filas Total
</commit_message>
<xml_diff>
--- a/ventas_ficticias_Q1_2026.xlsx
+++ b/ventas_ficticias_Q1_2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\INFORMATICA\Desktop\prueba\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2B6567C-64F7-4F5A-A6C1-9AF274914CB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{713B0EE1-E605-45AE-9C1C-1246D7940CF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="30">
   <si>
     <t>Concepto</t>
   </si>
@@ -118,9 +118,6 @@
   </si>
   <si>
     <t>Servicio de instalación</t>
-  </si>
-  <si>
-    <t>31/04/2026</t>
   </si>
 </sst>
 </file>
@@ -2266,7 +2263,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7875F631-FE92-4E7E-8946-FDF27C28EBB3}">
-  <dimension ref="A1:D42"/>
+  <dimension ref="A1:D40"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31.5703125" customWidth="1"/>
@@ -2348,165 +2345,165 @@
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="8" t="s">
-        <v>30</v>
+      <c r="B6" s="8">
+        <v>46141</v>
       </c>
       <c r="C6" s="4">
-        <v>4396.7299999999996</v>
+        <v>579.83000000000004</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>4</v>
+        <v>29</v>
       </c>
       <c r="B7" s="8">
-        <v>46141</v>
+        <v>46121</v>
       </c>
       <c r="C7" s="4">
-        <v>579.83000000000004</v>
+        <v>1444.69</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="B8" s="8">
-        <v>46121</v>
+        <v>46119</v>
       </c>
       <c r="C8" s="4">
-        <v>1444.69</v>
+        <v>3453.11</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="B9" s="8">
-        <v>46119</v>
+        <v>46128</v>
       </c>
       <c r="C9" s="4">
-        <v>3453.11</v>
+        <v>1293.05</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="B10" s="8">
-        <v>46128</v>
+        <v>46133</v>
       </c>
       <c r="C10" s="4">
-        <v>1293.05</v>
+        <v>2146.6999999999998</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="B11" s="8">
-        <v>46133</v>
+        <v>46113</v>
       </c>
       <c r="C11" s="4">
-        <v>2146.6999999999998</v>
+        <v>1701.1</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="B12" s="8">
-        <v>46113</v>
+        <v>46118</v>
       </c>
       <c r="C12" s="4">
-        <v>1701.1</v>
+        <v>3719.09</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="B13" s="8">
-        <v>46118</v>
+        <v>46130</v>
       </c>
       <c r="C13" s="4">
-        <v>3719.09</v>
+        <v>97.87</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="B14" s="8">
         <v>46130</v>
       </c>
       <c r="C14" s="4">
-        <v>97.87</v>
+        <v>228.34</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B15" s="8">
         <v>46130</v>
       </c>
       <c r="C15" s="4">
-        <v>228.34</v>
+        <v>783.06</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="B16" s="8">
-        <v>46130</v>
+        <v>46122</v>
       </c>
       <c r="C16" s="4">
-        <v>783.06</v>
+        <v>1855.04</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B17" s="8">
-        <v>46122</v>
+        <v>46119</v>
       </c>
       <c r="C17" s="4">
-        <v>1855.04</v>
+        <v>3426.23</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>9</v>
@@ -2517,108 +2514,108 @@
         <v>15</v>
       </c>
       <c r="B18" s="8">
-        <v>46119</v>
+        <v>46137</v>
       </c>
       <c r="C18" s="4">
-        <v>3426.23</v>
+        <v>2821.42</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="B19" s="8">
-        <v>46137</v>
+        <v>46136</v>
       </c>
       <c r="C19" s="4">
-        <v>2821.42</v>
+        <v>815.04</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B20" s="8">
-        <v>46136</v>
+        <v>46138</v>
       </c>
       <c r="C20" s="4">
-        <v>815.04</v>
+        <v>4063.32</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="B21" s="8">
-        <v>46138</v>
+        <v>46118</v>
       </c>
       <c r="C21" s="4">
-        <v>4063.32</v>
+        <v>3695.99</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B22" s="8">
-        <v>46118</v>
+        <v>46138</v>
       </c>
       <c r="C22" s="4">
-        <v>3695.99</v>
+        <v>3366.04</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="B23" s="8">
-        <v>46138</v>
+        <v>46118</v>
       </c>
       <c r="C23" s="4">
-        <v>3366.04</v>
+        <v>3947.5</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B24" s="8">
-        <v>46118</v>
+        <v>46140</v>
       </c>
       <c r="C24" s="4">
-        <v>3947.5</v>
+        <v>241.69</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="B25" s="8">
-        <v>46140</v>
+        <v>46119</v>
       </c>
       <c r="C25" s="4">
-        <v>241.69</v>
+        <v>4092.1</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>13</v>
@@ -2626,83 +2623,83 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="B26" s="8">
-        <v>46119</v>
+        <v>46122</v>
       </c>
       <c r="C26" s="4">
-        <v>4092.1</v>
+        <v>4111.66</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="B27" s="8">
-        <v>46122</v>
+        <v>46113</v>
       </c>
       <c r="C27" s="4">
-        <v>4111.66</v>
+        <v>3317.16</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="B28" s="8">
-        <v>46113</v>
+        <v>46121</v>
       </c>
       <c r="C28" s="4">
-        <v>3317.16</v>
+        <v>4328.55</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B29" s="8">
-        <v>46121</v>
+        <v>46133</v>
       </c>
       <c r="C29" s="4">
-        <v>4328.55</v>
+        <v>2571.56</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="B30" s="8">
-        <v>46133</v>
+        <v>46131</v>
       </c>
       <c r="C30" s="4">
-        <v>2571.56</v>
+        <v>4814.54</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B31" s="8" t="s">
-        <v>30</v>
+        <v>17</v>
+      </c>
+      <c r="B31" s="8">
+        <v>46116</v>
       </c>
       <c r="C31" s="4">
-        <v>186.62</v>
+        <v>3004.04</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>12</v>
@@ -2710,55 +2707,55 @@
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="B32" s="8">
-        <v>46131</v>
+        <v>46126</v>
       </c>
       <c r="C32" s="4">
-        <v>4814.54</v>
+        <v>3050.73</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="B33" s="8">
-        <v>46116</v>
+        <v>46125</v>
       </c>
       <c r="C33" s="4">
-        <v>3004.04</v>
+        <v>4502.55</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="B34" s="8">
-        <v>46126</v>
+        <v>46114</v>
       </c>
       <c r="C34" s="4">
-        <v>3050.73</v>
+        <v>3558.49</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="B35" s="8">
-        <v>46125</v>
+        <v>46142</v>
       </c>
       <c r="C35" s="4">
-        <v>4502.55</v>
+        <v>4042.23</v>
       </c>
       <c r="D35" s="2" t="s">
         <v>5</v>
@@ -2766,96 +2763,68 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="B36" s="8">
-        <v>46114</v>
+        <v>46126</v>
       </c>
       <c r="C36" s="4">
-        <v>3558.49</v>
+        <v>396.37</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B37" s="8">
-        <v>46142</v>
+        <v>46123</v>
       </c>
       <c r="C37" s="4">
-        <v>4042.23</v>
+        <v>3333.77</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="B38" s="8">
-        <v>46126</v>
+        <v>46129</v>
       </c>
       <c r="C38" s="4">
-        <v>396.37</v>
+        <v>1580.96</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="B39" s="8">
-        <v>46123</v>
+        <v>46125</v>
       </c>
       <c r="C39" s="4">
-        <v>3333.77</v>
+        <v>3501.18</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B40" s="8">
-        <v>46129</v>
-      </c>
-      <c r="C40" s="4">
-        <v>1580.96</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B41" s="8">
-        <v>46125</v>
-      </c>
-      <c r="C41" s="4">
-        <v>3501.18</v>
-      </c>
-      <c r="D41" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="5" t="s">
+      <c r="A40" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B42"/>
-      <c r="C42" s="6">
-        <f>SUM(C2:C41)</f>
-        <v>106240.79999999999</v>
+      <c r="B40"/>
+      <c r="C40" s="6">
+        <f>SUM(C2:C39)</f>
+        <v>101657.45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Agregar grafica Top Categorias mas vendidas
</commit_message>
<xml_diff>
--- a/ventas_ficticias_Q1_2026.xlsx
+++ b/ventas_ficticias_Q1_2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\INFORMATICA\Desktop\prueba\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{713B0EE1-E605-45AE-9C1C-1246D7940CF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89825D38-24F5-4C45-B5CE-969D9EE122F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -180,7 +180,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -199,6 +199,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2263,7 +2264,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7875F631-FE92-4E7E-8946-FDF27C28EBB3}">
-  <dimension ref="A1:D40"/>
+  <dimension ref="A1:E54"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31.5703125" customWidth="1"/>
@@ -2827,6 +2828,9 @@
         <v>101657.45</v>
       </c>
     </row>
+    <row r="54" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E54" s="10"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>